<commit_message>
Avance: Teoría de la información
Hice un programa de canales.
- Recibe entrada de frecuencias
- Recibe entrada de alfabeto
- Calcula frecuencias de salida
- Calcula Autoinformación
- Calcula Entropía
- Calcula Capacidad del canal
</commit_message>
<xml_diff>
--- a/Teoría de la información/1924910-Crema-4N1-MC/1924910-Crema-4N1-MC.xlsx
+++ b/Teoría de la información/1924910-Crema-4N1-MC/1924910-Crema-4N1-MC.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="A:\Repositorios\Semestre-EneJun2026\Teoría de la información\1924910-Crema-4N1-MC\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C68229A-9B1F-49B2-8659-FAD3AB575302}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1227C060-FCC8-4350-8334-790A166C9988}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12216" activeTab="1" xr2:uid="{90F7E246-578B-4CCA-9328-F46E37544E22}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="20376" windowHeight="12216" xr2:uid="{90F7E246-578B-4CCA-9328-F46E37544E22}"/>
   </bookViews>
   <sheets>
     <sheet name="Problema 2" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
   <si>
     <t>Matrícula:</t>
   </si>
@@ -62,9 +62,6 @@
   </si>
   <si>
     <t>Matríz de Transmisión</t>
-  </si>
-  <si>
-    <t>&lt;</t>
   </si>
   <si>
     <t>Frecuencia de salida</t>
@@ -297,15 +294,6 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -319,6 +307,15 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -743,302 +740,303 @@
       <c r="G6" s="5"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A7" s="7" t="s">
+      <c r="A7" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="8"/>
-      <c r="H7" s="9" t="s">
+      <c r="B7" s="17"/>
+      <c r="C7" s="17"/>
+      <c r="D7" s="17"/>
+      <c r="E7" s="17"/>
+      <c r="F7" s="7"/>
+      <c r="H7" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="I7" s="10" t="s">
+      <c r="I7" s="19" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="11" t="s">
+      <c r="A8" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="12"/>
-      <c r="C8" s="12" t="s">
+      <c r="B8" s="9"/>
+      <c r="C8" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F8" s="12"/>
-      <c r="H8" s="9"/>
-      <c r="I8" s="10"/>
+      <c r="F8" s="9"/>
+      <c r="H8" s="18"/>
+      <c r="I8" s="19"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
+      <c r="A9" s="10">
         <v>0.17</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C9" s="14">
+      <c r="C9" s="11">
         <v>0.98</v>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="E9" s="14">
+      <c r="E9" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="F9" s="14">
+      <c r="F9" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="G9" s="15"/>
-      <c r="H9" s="14">
+      <c r="G9" s="12"/>
+      <c r="H9" s="11">
         <f>-LOG(C9, 2)</f>
         <v>2.9146345659516508E-2</v>
       </c>
-      <c r="I9" s="13">
+      <c r="I9" s="10">
         <f>H9 * C9</f>
         <v>2.8563418746326178E-2</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A10" s="13">
+      <c r="A10" s="10">
         <v>0.38</v>
       </c>
-      <c r="B10" s="12" t="s">
+      <c r="B10" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C10" s="14">
+      <c r="C10" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="11">
         <v>0.98</v>
       </c>
-      <c r="E10" s="14">
+      <c r="E10" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="F10" s="14">
+      <c r="F10" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="H10" s="14">
+      <c r="H10" s="11">
         <f>-LOG(C10, 2)</f>
         <v>7.2288186904958796</v>
       </c>
-      <c r="I10" s="13">
+      <c r="I10" s="10">
         <f>H10 * C10</f>
         <v>4.8192124603305901E-2</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A11" s="13">
+      <c r="A11" s="10">
         <v>0.2</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="14">
+      <c r="C11" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="E11" s="14">
+      <c r="E11" s="11">
         <v>0.98</v>
       </c>
-      <c r="F11" s="14">
+      <c r="F11" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="H11" s="14">
+      <c r="H11" s="11">
         <f>-LOG(C11, 2)</f>
         <v>7.2288186904958796</v>
       </c>
-      <c r="I11" s="13">
+      <c r="I11" s="10">
         <f>H11 * C11</f>
         <v>4.8192124603305901E-2</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A12" s="13">
+      <c r="A12" s="10">
         <f>1 - (SUM(A9:A11))</f>
         <v>0.25</v>
       </c>
-      <c r="B12" s="12" t="s">
+      <c r="B12" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C12" s="14">
+      <c r="C12" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="D12" s="14">
+      <c r="D12" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="E12" s="14">
+      <c r="E12" s="11">
         <f>(1 - $C$9) / 3</f>
         <v>6.6666666666666723E-3</v>
       </c>
-      <c r="F12" s="14">
+      <c r="F12" s="11">
         <v>0.98</v>
       </c>
-      <c r="H12" s="14">
+      <c r="H12" s="11">
         <f>-LOG(C12, 2)</f>
         <v>7.2288186904958796</v>
       </c>
-      <c r="I12" s="13">
+      <c r="I12" s="10">
         <f>H12 * C12</f>
         <v>4.8192124603305901E-2</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="H13" s="16">
+      <c r="H13" s="13">
         <f>SUM(H9:H11)</f>
         <v>14.486783726651275</v>
       </c>
-      <c r="I13" s="17">
+      <c r="I13" s="14">
         <f>SUM(I9:I12)</f>
         <v>0.1731397925562439</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B14" s="7" t="s">
+      <c r="B14" s="17" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="8"/>
+      <c r="C14" s="17"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="7"/>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B15" s="12"/>
-      <c r="C15" s="12" t="s">
+      <c r="B15" s="9"/>
+      <c r="C15" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="E15" s="12" t="s">
+      <c r="E15" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" s="9" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="C16" s="14">
-        <f>C9 * $A9</f>
+      <c r="C16" s="11">
+        <f t="shared" ref="C16:F19" si="1">C9 * $A9</f>
         <v>0.1666</v>
       </c>
-      <c r="D16" s="14">
-        <f>D9 * $A9</f>
+      <c r="D16" s="11">
+        <f t="shared" si="1"/>
         <v>1.1333333333333343E-3</v>
       </c>
-      <c r="E16" s="14">
-        <f>E9 * $A9</f>
+      <c r="E16" s="11">
+        <f t="shared" si="1"/>
         <v>1.1333333333333343E-3</v>
       </c>
-      <c r="F16" s="14" t="s">
-        <v>12</v>
-      </c>
-      <c r="G16" s="15"/>
+      <c r="F16" s="11">
+        <f t="shared" si="1"/>
+        <v>1.1333333333333343E-3</v>
+      </c>
+      <c r="G16" s="12"/>
     </row>
     <row r="17" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B17" s="12" t="s">
+      <c r="B17" s="9" t="s">
         <v>3</v>
       </c>
-      <c r="C17" s="14">
-        <f>C10 * $A10</f>
+      <c r="C17" s="11">
+        <f t="shared" si="1"/>
         <v>2.5333333333333354E-3</v>
       </c>
-      <c r="D17" s="14">
-        <f>D10 * $A10</f>
+      <c r="D17" s="11">
+        <f t="shared" si="1"/>
         <v>0.37240000000000001</v>
       </c>
-      <c r="E17" s="14">
-        <f>E10 * $A10</f>
+      <c r="E17" s="11">
+        <f t="shared" si="1"/>
         <v>2.5333333333333354E-3</v>
       </c>
-      <c r="F17" s="14">
+      <c r="F17" s="11">
         <f>F10 * $A10</f>
         <v>2.5333333333333354E-3</v>
       </c>
     </row>
     <row r="18" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B18" s="12" t="s">
+      <c r="B18" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C18" s="14">
-        <f>C11 * $A11</f>
+      <c r="C18" s="11">
+        <f t="shared" si="1"/>
         <v>1.3333333333333346E-3</v>
       </c>
-      <c r="D18" s="14">
-        <f>D11 * $A11</f>
+      <c r="D18" s="11">
+        <f t="shared" si="1"/>
         <v>1.3333333333333346E-3</v>
       </c>
-      <c r="E18" s="14">
-        <f>E11 * $A11</f>
+      <c r="E18" s="11">
+        <f t="shared" si="1"/>
         <v>0.19600000000000001</v>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="11">
         <f>F11 * $A11</f>
         <v>1.3333333333333346E-3</v>
       </c>
     </row>
     <row r="19" spans="2:6" x14ac:dyDescent="0.3">
-      <c r="B19" s="12" t="s">
+      <c r="B19" s="9" t="s">
         <v>5</v>
       </c>
-      <c r="C19" s="14">
-        <f>C12 * $A12</f>
+      <c r="C19" s="11">
+        <f t="shared" si="1"/>
         <v>1.6666666666666681E-3</v>
       </c>
-      <c r="D19" s="14">
-        <f>D12 * $A12</f>
+      <c r="D19" s="11">
+        <f t="shared" si="1"/>
         <v>1.6666666666666681E-3</v>
       </c>
-      <c r="E19" s="14">
-        <f>E12 * $A12</f>
+      <c r="E19" s="11">
+        <f t="shared" si="1"/>
         <v>1.6666666666666681E-3</v>
       </c>
-      <c r="F19" s="14">
+      <c r="F19" s="11">
         <f>F12 * $A12</f>
         <v>0.245</v>
       </c>
     </row>
     <row r="20" spans="2:6" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="B20" s="18" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="19">
+      <c r="B20" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C20" s="16">
         <f>SUM(C16:C18)</f>
         <v>0.17046666666666666</v>
       </c>
-      <c r="D20" s="19">
+      <c r="D20" s="16">
         <f>SUM(D16:D18)</f>
         <v>0.37486666666666668</v>
       </c>
-      <c r="E20" s="19">
+      <c r="E20" s="16">
         <f>SUM(E16:E18)</f>
         <v>0.19966666666666669</v>
       </c>
-      <c r="F20" s="19">
+      <c r="F20" s="16">
         <f>SUM(F16:F18)</f>
-        <v>3.8666666666666702E-3</v>
+        <v>5.0000000000000044E-3</v>
       </c>
     </row>
   </sheetData>
@@ -1062,18 +1060,18 @@
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>15</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>16</v>
-      </c>
-      <c r="D3" t="s">
-        <v>17</v>
       </c>
       <c r="E3" t="s">
         <v>10</v>
@@ -1081,7 +1079,7 @@
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C4">
         <v>59928</v>
@@ -1097,7 +1095,7 @@
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C5">
         <v>59929</v>
@@ -1111,12 +1109,12 @@
         <v>0.15941641095851508</v>
       </c>
       <c r="G5" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B6" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C6">
         <v>60316</v>
@@ -1130,12 +1128,12 @@
         <v>0.16014542170424115</v>
       </c>
       <c r="G6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C7">
         <v>120814</v>
@@ -1151,7 +1149,7 @@
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <v>60025</v>
@@ -1167,7 +1165,7 @@
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C9">
         <v>60033</v>
@@ -1183,7 +1181,7 @@
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10">
         <v>120317</v>
@@ -1199,7 +1197,7 @@
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11">
         <v>60137</v>
@@ -1215,7 +1213,7 @@
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B12" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C12">
         <v>120309</v>
@@ -1231,7 +1229,7 @@
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B13" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C13">
         <v>119627</v>
@@ -1247,7 +1245,7 @@
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B14" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C14">
         <v>120048</v>
@@ -1263,7 +1261,7 @@
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B15" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C15">
         <v>120748</v>
@@ -1279,7 +1277,7 @@
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B16" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C16">
         <v>120423</v>
@@ -1295,7 +1293,7 @@
     </row>
     <row r="17" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B17" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C17">
         <v>59921</v>
@@ -1311,7 +1309,7 @@
     </row>
     <row r="18" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C18">
         <v>120108</v>
@@ -1327,7 +1325,7 @@
     </row>
     <row r="19" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C19">
         <v>60041</v>
@@ -1343,7 +1341,7 @@
     </row>
     <row r="20" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B20" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C20">
         <v>60115</v>
@@ -1359,7 +1357,7 @@
     </row>
     <row r="21" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B21" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C21">
         <v>120168</v>
@@ -1375,7 +1373,7 @@
     </row>
     <row r="22" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B22" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C22">
         <v>59955</v>
@@ -1391,7 +1389,7 @@
     </row>
     <row r="23" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B23" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C23">
         <v>121127</v>
@@ -1407,7 +1405,7 @@
     </row>
     <row r="24" spans="2:5" x14ac:dyDescent="0.3">
       <c r="B24" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C24">
         <v>60229</v>

</xml_diff>